<commit_message>
docs(reports): deploy unified consolidated summary reports for build 18
</commit_message>
<xml_diff>
--- a/reports/history/android/build-18/Excel/Failed_Test_Cases.xlsx
+++ b/reports/history/android/build-18/Excel/Failed_Test_Cases.xlsx
@@ -482,12 +482,12 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="9568" customWidth="1" min="8" max="8"/>
+    <col width="9450" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -543,7 +543,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TC_GEN_004</t>
+          <t>TC_GEN_001</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>test_market_prices_page_load</t>
+          <t>test_auth_client_validation</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -568,29 +568,27 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>32.67</t>
+          <t>37.13</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 07:38:22</t>
+          <t>2026-06-24 01:02:14</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>driver = &lt;appium.webdriver.webdriver.WebDriver (session="ba4e3fe3-70e3-4cf3-a74e-efc34d87a79e")&gt;
-    @pytest.fixture(scope="function")
-    def auth_driver(driver):
-        """Fixture to launch app and log in automatically with test credentials."""
-        time.sleep(5)
+          <t>driver = &lt;appium.webdriver.webdriver.WebDriver (session="00625872-fc8f-4afa-8e82-501673e0c66e")&gt;
+    def test_auth_client_validation(driver):
+        """Test that login validation fails when submitting empty fields on mobile."""
+        time.sleep(5)  # Wait for app to boot on emulator
         login_page = LoginPage(driver)
-        print("[MobileTest] Performing E2E test login...")
-&gt;       login_page.login("testfarmer@example.com", "TestFarmer123!")
-tests/mobile_e2e/test_suites/test_features.py:14: 
+        login_page.capture_screenshot("mobile_login_screen_load")
+        # Submit empty fields
+&gt;       login_page.click(login_page.SUBMIT_BUTTON)
+tests/mobile_e2e/test_suites/test_auth.py:12: 
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ 
-tests/mobile_e2e/pages/login_page.py:14: in login
-    self.send_keys(self.EMAIL_INPUT, email)
-tests/mobile_e2e/pages/base_page.py:31: in send_keys
+tests/mobile_e2e/pages/base_page.py:26: in click
     element = self.wait_for_element(locator)
               ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
 tests/mobile_e2e/pages/base_page.py:22: in wait_for_element
@@ -609,8 +607,8 @@
 /opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/remote/webdriver.py:492: in execute
     self.error_handler.check_response(response)
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ 
-self = &lt;appium.webdriver.errorhandler.MobileErrorHandler object at 0x7f4d0b376f90&gt;
-response = {'status': 500, 'value': '{"value":{"error":"unknown error","message":"Timed out after 10505ms waiting for the root Ac...r2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath2(AccessibilityNodeInfoDumper.java:327)\\n\\t... 33 more\\n"}}'}
+self = &lt;appium.webdriver.errorhandler.MobileErrorHandler object at 0x7fc0b4b71310&gt;
+response = {'status': 500, 'value': '{"value":{"error":"unknown error","message":"io.appium.uiautomator2.common.exceptions.UiAuto...r2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:279)\\n\\t... 33 more\\n"}}'}
     def check_response(self, response: Dict[str, Any]) -&gt; None:
         """
         https://www.w3.org/TR/webdriver/#errors
@@ -651,11 +649,11 @@
                 alert_text=value.get('data'),
             )
 &gt;       raise exception_class(msg=message, stacktrace=format_stacktrace(stacktrace))
-E       selenium.common.exceptions.WebDriverException: Message: Timed out after 10505ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work. Try changing the 'enforceXPath1' driver setting to 'true' in order to workaround the problem.
+E       selenium.common.exceptions.WebDriverException: Message: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
 E       Stacktrace:
-E       io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10505ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work. Try changing the 'enforceXPath1' driver setting to 'true' in order to workaround the problem.
-E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath2(AccessibilityNodeInfoDumper.java:366)
-E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodes(AccessibilityNodeInfoDumper.java:378)
+E       io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:306)
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodes(AccessibilityNodeInfoDumper.java:377)
 E       	at io.appium.uiautomator2.utils.ElementLocationHelpers.getXPathNodeMatch(ElementLocationHelpers.java:124)
 E       	at io.appium.uiautomator2.utils.ElementLocationHelpers.findElement(ElementLocationHelpers.java:151)
 E       	at io.appium.uiautomator2.handler.FindElement.safeHandle(FindElement.java:60)
@@ -688,12 +686,12 @@
 E       	at io.netty.util.internal.ThreadExecutorMap$2.run(ThreadExecutorMap.java:74)
 E       	at io.netty.util.concurrent.FastThreadLocalRunnable.run(FastThreadLocalRunnable.java:30)
 E       	at java.lang.Thread.run(Thread.java:919)
-E       Caused by: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10505ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
+E       Caused by: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
 E       	at io.appium.uiautomator2.utils.AXWindowHelpers.getActiveWindowRoot(AXWindowHelpers.java:107)
 E       	at io.appium.uiautomator2.utils.AXWindowHelpers.retrieveWindowRoots(AXWindowHelpers.java:87)
 E       	at io.appium.uiautomator2.utils.AXWindowHelpers.getCachedWindowRoots(AXWindowHelpers.java:68)
 E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.toStream(AccessibilityNodeInfoDumper.java:228)
-E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath2(AccessibilityNodeInfoDumper.java:327)
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:279)
 E       	... 33 more
 /opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/appium/webdriver/errorhandler.py:125: WebDriverException</t>
         </is>

</xml_diff>